<commit_message>
feat(nrw): snap report period to Nepali (BS) months and read SCADA layout-independently
- auto-set the date range to the BS month a SCADA workbook covers instead of the raw file span, so consumption and supply span the same billing month
- locate SCADA sheets by their 'Day' header row and customer columns by header name, with fallbacks to the canonical layout
- match 'dma 9.1' style names against plain '9.1 (OMU 036)' headers; list available DMA columns when a lookup fails
- show period label, days found vs. requested, and warn when missing SCADA days under-count supplied water
- reset restores the default date range; bump nrw-builder to v9 and the service worker cache
</commit_message>
<xml_diff>
--- a/website/DMA wise area allocation.xlsx
+++ b/website/DMA wise area allocation.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Intern\website\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C83010C3-A236-4C5D-8478-180EB4FA1AC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E91FFE6-5C95-42FB-B046-3D1CA1421E7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-109" yWindow="-109" windowWidth="26301" windowHeight="14889" xr2:uid="{42E43884-7973-4028-8C7B-2B70ABE36626}"/>
   </bookViews>
@@ -180,20 +180,20 @@
     <t>32G</t>
   </si>
   <si>
-    <t>18-29</t>
-  </si>
-  <si>
     <t>32e</t>
   </si>
   <si>
     <t>35a</t>
+  </si>
+  <si>
+    <t>19-29</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -208,17 +208,23 @@
       <family val="2"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
+      <sz val="16"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
     <font>
-      <sz val="16"/>
+      <b/>
+      <sz val="11"/>
       <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -380,26 +386,26 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
@@ -726,398 +732,398 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="21.1" x14ac:dyDescent="0.35">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="14.3" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:4" ht="14.3" x14ac:dyDescent="0.25">
-      <c r="A4" s="10" t="s">
+      <c r="A4" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="11" t="s">
+      <c r="B4" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="11" t="s">
+      <c r="C4" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="12" t="s">
+      <c r="D4" s="6" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" s="3"/>
+    <row r="5" spans="1:4" ht="14.3" x14ac:dyDescent="0.25">
+      <c r="A5" s="7"/>
       <c r="B5" s="16">
         <v>1.2</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="9" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A6" s="3"/>
+    <row r="6" spans="1:4" ht="14.3" x14ac:dyDescent="0.25">
+      <c r="A6" s="7"/>
       <c r="B6" s="16"/>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="9" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A7" s="3"/>
-      <c r="B7" s="6">
+    <row r="7" spans="1:4" ht="14.3" x14ac:dyDescent="0.25">
+      <c r="A7" s="7"/>
+      <c r="B7" s="10">
         <v>2.1</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="D7" s="9" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A8" s="3"/>
+    <row r="8" spans="1:4" ht="14.3" x14ac:dyDescent="0.25">
+      <c r="A8" s="7"/>
       <c r="B8" s="14">
         <v>2.2000000000000002</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="D8" s="9" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A9" s="3"/>
+    <row r="9" spans="1:4" ht="14.3" x14ac:dyDescent="0.25">
+      <c r="A9" s="7"/>
       <c r="B9" s="14"/>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="D9" s="9" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A10" s="3"/>
+    <row r="10" spans="1:4" ht="14.3" x14ac:dyDescent="0.25">
+      <c r="A10" s="7"/>
       <c r="B10" s="14"/>
-      <c r="C10" s="4" t="s">
+      <c r="C10" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="D10" s="5" t="s">
+      <c r="D10" s="9" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A11" s="3"/>
+    <row r="11" spans="1:4" ht="14.3" x14ac:dyDescent="0.25">
+      <c r="A11" s="7"/>
       <c r="B11" s="14"/>
-      <c r="C11" s="4" t="s">
+      <c r="C11" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="D11" s="5" t="s">
+      <c r="D11" s="9" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A12" s="3"/>
-      <c r="B12" s="6">
+    <row r="12" spans="1:4" ht="14.3" x14ac:dyDescent="0.25">
+      <c r="A12" s="7"/>
+      <c r="B12" s="10">
         <v>2.2999999999999998</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="C12" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="D12" s="5" t="s">
+      <c r="D12" s="9" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A13" s="3"/>
+    <row r="13" spans="1:4" ht="14.3" x14ac:dyDescent="0.25">
+      <c r="A13" s="7"/>
       <c r="B13" s="14">
         <v>2.4</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="C13" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="D13" s="5" t="s">
+      <c r="D13" s="9" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A14" s="3"/>
+    <row r="14" spans="1:4" ht="14.3" x14ac:dyDescent="0.25">
+      <c r="A14" s="7"/>
       <c r="B14" s="14"/>
-      <c r="C14" s="4" t="s">
+      <c r="C14" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="D14" s="5" t="s">
+      <c r="D14" s="9" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A15" s="3"/>
+    <row r="15" spans="1:4" ht="14.3" x14ac:dyDescent="0.25">
+      <c r="A15" s="7"/>
       <c r="B15" s="14"/>
-      <c r="C15" s="4" t="s">
+      <c r="C15" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="D15" s="5" t="s">
+      <c r="D15" s="9" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A16" s="3"/>
+    <row r="16" spans="1:4" ht="14.3" x14ac:dyDescent="0.25">
+      <c r="A16" s="7"/>
       <c r="B16" s="14">
         <v>3.1</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="C16" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="D16" s="5" t="s">
+      <c r="D16" s="9" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A17" s="3"/>
+    <row r="17" spans="1:4" ht="14.3" x14ac:dyDescent="0.25">
+      <c r="A17" s="7"/>
       <c r="B17" s="14"/>
-      <c r="C17" s="4" t="s">
+      <c r="C17" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="D17" s="5" t="s">
+      <c r="D17" s="9" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A18" s="3"/>
+    <row r="18" spans="1:4" ht="14.3" x14ac:dyDescent="0.25">
+      <c r="A18" s="7"/>
       <c r="B18" s="14">
         <v>3.2</v>
       </c>
-      <c r="C18" s="4" t="s">
+      <c r="C18" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="D18" s="5" t="s">
+      <c r="D18" s="9" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A19" s="3"/>
+    <row r="19" spans="1:4" ht="14.3" x14ac:dyDescent="0.25">
+      <c r="A19" s="7"/>
       <c r="B19" s="14"/>
-      <c r="C19" s="4" t="s">
+      <c r="C19" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="D19" s="5" t="s">
+      <c r="D19" s="9" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A20" s="3"/>
+    <row r="20" spans="1:4" ht="14.3" x14ac:dyDescent="0.25">
+      <c r="A20" s="7"/>
       <c r="B20" s="14">
         <v>3.3</v>
       </c>
-      <c r="C20" s="4" t="s">
+      <c r="C20" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="D20" s="5" t="s">
+      <c r="D20" s="9" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A21" s="3"/>
+    <row r="21" spans="1:4" ht="14.3" x14ac:dyDescent="0.25">
+      <c r="A21" s="7"/>
       <c r="B21" s="14"/>
-      <c r="C21" s="4" t="s">
+      <c r="C21" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="D21" s="5" t="s">
+      <c r="D21" s="9" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A22" s="3"/>
+    <row r="22" spans="1:4" ht="14.3" x14ac:dyDescent="0.25">
+      <c r="A22" s="7"/>
       <c r="B22" s="14"/>
-      <c r="C22" s="4" t="s">
+      <c r="C22" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="D22" s="5" t="s">
+      <c r="D22" s="9" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A23" s="3"/>
+    <row r="23" spans="1:4" ht="14.3" x14ac:dyDescent="0.25">
+      <c r="A23" s="7"/>
       <c r="B23" s="14"/>
-      <c r="C23" s="4" t="s">
+      <c r="C23" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="D23" s="5" t="s">
+      <c r="D23" s="9" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A24" s="3"/>
+    <row r="24" spans="1:4" ht="14.3" x14ac:dyDescent="0.25">
+      <c r="A24" s="7"/>
       <c r="B24" s="14"/>
-      <c r="C24" s="4" t="s">
+      <c r="C24" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="D24" s="5" t="s">
+      <c r="D24" s="9" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A25" s="3"/>
+    <row r="25" spans="1:4" ht="14.3" x14ac:dyDescent="0.25">
+      <c r="A25" s="7"/>
       <c r="B25" s="14">
         <v>3.4</v>
       </c>
-      <c r="C25" s="4" t="s">
+      <c r="C25" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="D25" s="5" t="s">
+      <c r="D25" s="9" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A26" s="3"/>
+    <row r="26" spans="1:4" ht="14.3" x14ac:dyDescent="0.25">
+      <c r="A26" s="7"/>
       <c r="B26" s="14"/>
-      <c r="C26" s="4" t="s">
+      <c r="C26" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="D26" s="5" t="s">
+      <c r="D26" s="9" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A27" s="3"/>
+    <row r="27" spans="1:4" ht="14.3" x14ac:dyDescent="0.25">
+      <c r="A27" s="7"/>
       <c r="B27" s="14"/>
-      <c r="C27" s="4" t="s">
+      <c r="C27" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="D27" s="5" t="s">
+      <c r="D27" s="9" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A28" s="3"/>
+    <row r="28" spans="1:4" ht="14.3" x14ac:dyDescent="0.25">
+      <c r="A28" s="7"/>
       <c r="B28" s="14">
         <v>3.5</v>
       </c>
-      <c r="C28" s="4" t="s">
+      <c r="C28" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="D28" s="5" t="s">
+      <c r="D28" s="9" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A29" s="3"/>
+    <row r="29" spans="1:4" ht="14.3" x14ac:dyDescent="0.25">
+      <c r="A29" s="7"/>
       <c r="B29" s="14"/>
-      <c r="C29" s="4" t="s">
+      <c r="C29" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="D29" s="5" t="s">
+      <c r="D29" s="9" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A30" s="3"/>
-      <c r="B30" s="6" t="s">
+    <row r="30" spans="1:4" ht="14.3" x14ac:dyDescent="0.25">
+      <c r="A30" s="7"/>
+      <c r="B30" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="C30" s="4" t="s">
+      <c r="C30" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="D30" s="5" t="s">
+      <c r="D30" s="9" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A31" s="3"/>
+    <row r="31" spans="1:4" ht="14.3" x14ac:dyDescent="0.25">
+      <c r="A31" s="7"/>
       <c r="B31" s="14">
         <v>9.1</v>
       </c>
-      <c r="C31" s="4" t="s">
+      <c r="C31" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="D31" s="5" t="s">
+      <c r="D31" s="9" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A32" s="3"/>
+    <row r="32" spans="1:4" ht="14.3" x14ac:dyDescent="0.25">
+      <c r="A32" s="7"/>
       <c r="B32" s="14"/>
-      <c r="C32" s="4" t="s">
+      <c r="C32" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="D32" s="5" t="s">
+      <c r="D32" s="9" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A33" s="3"/>
+    <row r="33" spans="1:4" ht="14.3" x14ac:dyDescent="0.25">
+      <c r="A33" s="7"/>
       <c r="B33" s="14"/>
-      <c r="C33" s="4" t="s">
+      <c r="C33" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="D33" s="5" t="s">
+      <c r="D33" s="9" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A34" s="3"/>
+    <row r="34" spans="1:4" ht="14.3" x14ac:dyDescent="0.25">
+      <c r="A34" s="7"/>
       <c r="B34" s="14"/>
-      <c r="C34" s="4" t="s">
+      <c r="C34" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="D34" s="5" t="s">
+      <c r="D34" s="9" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A35" s="3"/>
+    <row r="35" spans="1:4" ht="14.3" x14ac:dyDescent="0.25">
+      <c r="A35" s="7"/>
       <c r="B35" s="14">
         <v>9.1999999999999993</v>
       </c>
-      <c r="C35" s="4" t="s">
+      <c r="C35" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="D35" s="5" t="s">
+      <c r="D35" s="9" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A36" s="3"/>
+    <row r="36" spans="1:4" ht="14.3" x14ac:dyDescent="0.25">
+      <c r="A36" s="7"/>
       <c r="B36" s="14"/>
-      <c r="C36" s="4" t="s">
+      <c r="C36" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="D36" s="5" t="s">
+      <c r="D36" s="9" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" ht="14.3" x14ac:dyDescent="0.25">
+      <c r="A37" s="7"/>
+      <c r="B37" s="14"/>
+      <c r="C37" s="8" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A37" s="3"/>
-      <c r="B37" s="14"/>
-      <c r="C37" s="4" t="s">
+      <c r="D37" s="9" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" ht="14.3" x14ac:dyDescent="0.25">
+      <c r="A38" s="7"/>
+      <c r="B38" s="14"/>
+      <c r="C38" s="10">
+        <v>35</v>
+      </c>
+      <c r="D38" s="9" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" ht="14.95" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="11"/>
+      <c r="B39" s="15"/>
+      <c r="C39" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="D37" s="5" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A38" s="3"/>
-      <c r="B38" s="14"/>
-      <c r="C38" s="6">
-        <v>35</v>
-      </c>
-      <c r="D38" s="5" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" ht="14.3" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="7"/>
-      <c r="B39" s="15"/>
-      <c r="C39" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="D39" s="9" t="s">
+      <c r="D39" s="13" t="s">
         <v>11</v>
       </c>
     </row>

</xml_diff>